<commit_message>
Fix breadth so a holiday row is not stored as zero.
A VIX-only holiday was punching a hole through the 50-day average, and the missing readings were written as 0. Breadth now skips sessions where stocks did not trade, and a missing average stays blank. The Today file also counts BUY labels and leaves a column for the QQQ day change.

Co-authored-by: PatelNicknp <PatelNicknp@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Nick_Stock_Desk_Starter.xlsx
+++ b/data/Nick_Stock_Desk_Starter.xlsx
@@ -3677,7 +3677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3693,116 +3693,1689 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>qqq_day_pct</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>buy_count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>breadth_sma20</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>breadth_sma50</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>breadth_sma100</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>breadth_sma200</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>breadth_sma50_week_ago</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>advancers</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>decliners</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>universe_n</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>highs_52w</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>lows_52w</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>put_call</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>put_call_ma5</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>put_call_zone</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>put_call_name</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>vix</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>fred_dgs10</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>fred_t10y2y</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>xly_xlp</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>updated_pt</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>price_as_of</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>macro_growth</t>
+        </is>
+      </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>breadth_sma50</t>
+          <t>macro_inflation</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>breadth_sma100</t>
+          <t>macro_jobs</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>breadth_sma200</t>
+          <t>macro_score</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>breadth_sma50_week_ago</t>
+          <t>plain_english</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>advancers</t>
+          <t>data_status</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>decliners</t>
+          <t>note</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>universe_n</t>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>desk_median_trailing_pe</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>official_sp500_pe</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>official_status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>dist_52w_high_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>volume_ratio</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>note</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>highs_52w</t>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>trend_label</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>sma_alignment</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>above_sma20</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>above_sma50</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>above_sma100</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>above_sma200</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>score</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>lows_52w</t>
+          <t>data_status</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>put_call</t>
+          <t>note</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>put_call_ma5</t>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>rsi14</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>entry_low</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>entry_high</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>passes</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>why</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>side</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>day_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>day_pct</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>week_pct</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>month_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>month3_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ytd_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>pct_above_sma50</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>score_avg</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ret_1d</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ret_1w</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ret_1m</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ret_ytd</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>above_sma20</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>above_sma50</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>above_sma100</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>above_sma200</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n_missing</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n_present</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>latest</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>checked_pt</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>group_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>day_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>week_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>month_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>month3_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ytd_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>rs_3m_pct</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>score_avg</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>n_stocks</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>pct_above_sma50</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>macro_growth</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>macro_inflation</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>put_call_zone</t>
+          <t>macro_jobs</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>put_call_name</t>
+          <t>macro_score</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>vix</t>
+          <t>data_status</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>fred_dgs10</t>
+          <t>note</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>fred_t10y2y</t>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>plain_english</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>setting</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>sector</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>index_membership</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>in_sp500</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>in_ndx100</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>in_growth</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>window</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>top20_cagr_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>spy_cagr_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>bottom20_cagr_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>top20_total_pct</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>spy_total_pct</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>bottom20_total_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>top20_max_drawdown_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>spy_max_drawdown_pct</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>hit_rate_12w_pct</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>top_bucket_excess_12w_pct</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>headline</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>is_headline</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>horizon</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>bucket</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>avg_return_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>avg_spy_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>excess_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>hit_rate_pct</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>top20</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>spy</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>bottom20</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>top20_pct</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>spy_pct</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>difference_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>hit_rate_12w_pct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>signals</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>pct_above_sma20</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>pct_above_sma50</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>pct_above_sma100</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>pct_above_sma200</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>score_prev</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>verdict_prev</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>day_pct</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>score_prev</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>score_change</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>data_status</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>disclaimer</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ticker</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>company</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>shares</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>avg_cost</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>day_pct</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>gain</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>gain_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>weight_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>score_week_ago</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>score_week_change</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>verdict</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>stop</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>example</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>data_status</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>xly_xlp</t>
+          <t>note</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>updated_pt</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>price_as_of</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
           <t>disclaimer</t>
         </is>
       </c>
@@ -3810,1567 +5383,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>macro_growth</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>macro_inflation</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>macro_jobs</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>macro_score</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>plain_english</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>desk_median_trailing_pe</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>official_sp500_pe</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>official_status</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>dist_52w_high_pct</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>volume_ratio</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>trend_label</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>sma_alignment</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>above_sma20</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>above_sma50</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>above_sma100</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>above_sma200</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>rsi14</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>entry_low</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>entry_high</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>passes</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>why</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>side</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>day_pct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>day_pct</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>week_pct</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>month_pct</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>month3_pct</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ytd_pct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>pct_above_sma50</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>score_avg</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>ret_1d</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>ret_1w</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>ret_1m</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ret_ytd</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>above_sma20</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>above_sma50</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>above_sma100</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>above_sma200</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>field</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>n_missing</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>n_present</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>latest</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>checked_pt</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>group_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>day_pct</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>week_pct</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>month_pct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>month3_pct</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>ytd_pct</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>rs_3m_pct</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>score_avg</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>n_stocks</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>pct_above_sma50</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>macro_growth</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>macro_inflation</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>macro_jobs</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>macro_score</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>topic</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>plain_english</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>setting</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>sector</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>index_membership</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>in_sp500</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>in_ndx100</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>in_growth</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>window</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>start</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>end</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>top20_cagr_pct</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>spy_cagr_pct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>bottom20_cagr_pct</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>top20_total_pct</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>spy_total_pct</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>bottom20_total_pct</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>top20_max_drawdown_pct</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>spy_max_drawdown_pct</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>hit_rate_12w_pct</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>top_bucket_excess_12w_pct</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>headline</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>is_headline</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>horizon</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>bucket</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>avg_return_pct</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>avg_spy_pct</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>excess_pct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>hit_rate_pct</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet55.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>top20</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>spy</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>bottom20</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet56.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>top20_pct</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>spy_pct</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>difference_pct</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>hit_rate_12w_pct</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>signals</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet57.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>item</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>detail</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>pct_above_sma20</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>pct_above_sma50</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>pct_above_sma100</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>pct_above_sma200</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>kind</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>score_prev</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>verdict_prev</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>day_pct</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>score_prev</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>score_change</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:U1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>company</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>shares</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>avg_cost</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>price</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>day_pct</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>gain</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>gain_pct</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>weight_pct</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>score_week_ago</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>score_week_change</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>verdict</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>stop</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>example</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>data_status</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>disclaimer</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>